<commit_message>
Add document ownership (Product Owner / Product & Tech-Security Head) to compliance docs
- Inject accountable-roles block into Docs 01-04, 07-10 (Markdown + regenerated Word):
  Product Owner: Sridhar Muppidi; Product Head: Sachin Tulla; Technical & Security Head: Sachin Tulla.
- Annotate the three spreadsheets (05 SoA, 06 Evidence Pack, 07 tracker) with the same ownership line.
- Word-only document set (per request).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/compliance/05-Statement-of-Applicability.xlsx
+++ b/docs/compliance/05-Statement-of-Applicability.xlsx
@@ -484,7 +484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G98"/>
+  <dimension ref="A1:G100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3820,10 +3820,18 @@
       </c>
       <c r="G96" s="4" t="inlineStr"/>
     </row>
+    <row r="97"/>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
           <t>Note: control titles per ISO/IEC 27001:2022 Annex A — verify against the standard text. Status: Implemented / Partial / Planned / Inherited / Open.</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Document ownership — Product Owner: Sridhar Muppidi | Product Head: Sachin Tulla | Technical &amp; Security Head: Sachin Tulla</t>
         </is>
       </c>
     </row>

</xml_diff>